<commit_message>
fix: correct stale figures, pin snapshot date, reproducible workbook
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/costplus_suite/output/PBM_Markup_Analysis.xlsx
+++ b/costplus_suite/output/PBM_Markup_Analysis.xlsx
@@ -19,12 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0&quot;%&quot;"/>
-  </numFmts>
-  <fonts count="20">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,14 +34,6 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00404040"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <color rgb="00606060"/>
-      <sz val="10"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
@@ -56,64 +44,9 @@
       <sz val="14"/>
     </font>
     <font>
-      <sz val="11"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="000A0E1A"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <sz val="10"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="FF000080"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="FF006400"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="FF800080"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="FF8B0000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF006400"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF8B0000"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF800080"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF000080"/>
     </font>
   </fonts>
   <fills count="4">
@@ -126,11 +59,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000A0E1A"/>
+        <bgColor rgb="000A0E1A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -146,31 +81,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -554,118 +470,118 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PBM Markup Analysis — Generic Drug Overpayment vs Cost Plus Prices</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Estimated annual Medicare Part D + Medicaid overpayment. Generics only. Net prices never estimated.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>Data as of July 8, 2026 (most recent NADAC snapshot)</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Data as of July 16, 2026 (leaderboard.csv build time)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Source types (see METHODOLOGY.md for the selection-bias caveat):</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>federal_study — FTC interim reports (industry-wide sample)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>state_disclosure — Maine MHDO (mandated reporting)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>peer_reviewed — JAMA Mattingly (academic sample)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>litigation — J&amp;J and Wells Fargo ERISA complaints (plaintiff-selected, not representative)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Drug</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Cost Plus/unit</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>NADAC Acquisition/unit</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Medicare Pays/unit</t>
         </is>
       </c>
-      <c r="F10" s="19" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Gap/unit</t>
         </is>
       </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Total Overpayment</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Confirmed Markup %</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Estimated PBM Price/unit</t>
         </is>
       </c>
-      <c r="J10" s="19" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Source Citation</t>
         </is>
       </c>
-      <c r="K10" s="19" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Source Type</t>
         </is>
       </c>
-      <c r="L10" s="19" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
@@ -796,7 +712,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K14" s="20" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -902,7 +818,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K17" s="20" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -978,7 +894,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K19" s="20" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -1054,7 +970,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K21" s="20" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -1130,7 +1046,7 @@
           <t>FTC Second Interim Staff Report (Jan 2025), p.36</t>
         </is>
       </c>
-      <c r="K23" s="23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>federal_study</t>
         </is>
@@ -1440,7 +1356,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K33" s="20" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -1576,7 +1492,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K37" s="21" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -1622,7 +1538,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K38" s="20" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -2142,7 +2058,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K55" s="21" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -2416,7 +2332,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K64" s="20" t="inlineStr">
+      <c r="K64" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -2492,7 +2408,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K66" s="20" t="inlineStr">
+      <c r="K66" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -2946,7 +2862,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K81" s="20" t="inlineStr">
+      <c r="K81" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -4642,7 +4558,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.23</t>
         </is>
       </c>
-      <c r="K139" s="20" t="inlineStr">
+      <c r="K139" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -4712,7 +4628,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K141" s="21" t="inlineStr">
+      <c r="K141" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -4992,7 +4908,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K150" s="20" t="inlineStr">
+      <c r="K150" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -5272,7 +5188,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.23</t>
         </is>
       </c>
-      <c r="K159" s="20" t="inlineStr">
+      <c r="K159" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -5957,7 +5873,7 @@
           <t>JAMA Health Forum, Mattingly et al. (Oct 2023), p.2</t>
         </is>
       </c>
-      <c r="K182" s="22" t="inlineStr">
+      <c r="K182" t="inlineStr">
         <is>
           <t>peer_reviewed</t>
         </is>
@@ -6177,7 +6093,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K189" s="21" t="inlineStr">
+      <c r="K189" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -8329,7 +8245,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.23</t>
         </is>
       </c>
-      <c r="K264" s="20" t="inlineStr">
+      <c r="K264" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -8777,7 +8693,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K280" s="20" t="inlineStr">
+      <c r="K280" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -9951,7 +9867,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K321" s="21" t="inlineStr">
+      <c r="K321" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -10567,7 +10483,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.23</t>
         </is>
       </c>
-      <c r="K343" s="20" t="inlineStr">
+      <c r="K343" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -10709,7 +10625,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K348" s="21" t="inlineStr">
+      <c r="K348" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -10923,7 +10839,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K355" s="21" t="inlineStr">
+      <c r="K355" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -12217,7 +12133,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.23</t>
         </is>
       </c>
-      <c r="K401" s="20" t="inlineStr">
+      <c r="K401" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -12419,7 +12335,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K408" s="21" t="inlineStr">
+      <c r="K408" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -12489,7 +12405,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K410" s="20" t="inlineStr">
+      <c r="K410" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -12721,7 +12637,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K418" s="21" t="inlineStr">
+      <c r="K418" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -12983,7 +12899,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K427" s="20" t="inlineStr">
+      <c r="K427" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -13047,7 +12963,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K429" s="20" t="inlineStr">
+      <c r="K429" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -13945,7 +13861,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K461" s="21" t="inlineStr">
+      <c r="K461" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -14255,7 +14171,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K471" s="21" t="inlineStr">
+      <c r="K471" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -14943,7 +14859,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.23</t>
         </is>
       </c>
-      <c r="K495" s="20" t="inlineStr">
+      <c r="K495" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -15397,7 +15313,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K511" s="20" t="inlineStr">
+      <c r="K511" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -19637,7 +19553,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K666" s="21" t="inlineStr">
+      <c r="K666" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -23061,7 +22977,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.23</t>
         </is>
       </c>
-      <c r="K789" s="20" t="inlineStr">
+      <c r="K789" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -23125,7 +23041,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K791" s="21" t="inlineStr">
+      <c r="K791" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -23963,7 +23879,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K822" s="20" t="inlineStr">
+      <c r="K822" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -24297,7 +24213,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K834" s="20" t="inlineStr">
+      <c r="K834" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -24811,7 +24727,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K852" s="20" t="inlineStr">
+      <c r="K852" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -27065,7 +26981,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K934" s="20" t="inlineStr">
+      <c r="K934" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -27165,7 +27081,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K937" s="20" t="inlineStr">
+      <c r="K937" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -31879,7 +31795,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K1110" s="20" t="inlineStr">
+      <c r="K1110" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -35057,7 +34973,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K1226" s="21" t="inlineStr">
+      <c r="K1226" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -37809,7 +37725,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K1328" s="20" t="inlineStr">
+      <c r="K1328" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -38881,7 +38797,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K1366" s="20" t="inlineStr">
+      <c r="K1366" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -42185,7 +42101,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K1488" s="21" t="inlineStr">
+      <c r="K1488" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -43161,7 +43077,7 @@
           <t>Lewandowski v. Johnson &amp; Johnson, ERISA Class Action Complaint (D.N.J. 1:24-cv-00671, filed Feb. 2024), p.44</t>
         </is>
       </c>
-      <c r="K1522" s="21" t="inlineStr">
+      <c r="K1522" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -44671,7 +44587,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K1578" s="21" t="inlineStr">
+      <c r="K1578" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -46589,7 +46505,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K1650" s="21" t="inlineStr">
+      <c r="K1650" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -47889,7 +47805,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K1698" s="20" t="inlineStr">
+      <c r="K1698" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -52153,7 +52069,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K1858" s="21" t="inlineStr">
+      <c r="K1858" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -52367,7 +52283,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K1865" s="20" t="inlineStr">
+      <c r="K1865" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -52413,7 +52329,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.25</t>
         </is>
       </c>
-      <c r="K1866" s="20" t="inlineStr">
+      <c r="K1866" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -57037,7 +56953,7 @@
           <t>Navarro v. Wells Fargo &amp; Co., ERISA Class Action Complaint (D. Minn. 0:24-cv-03043, filed Jul. 2024), p.55</t>
         </is>
       </c>
-      <c r="K2037" s="21" t="inlineStr">
+      <c r="K2037" t="inlineStr">
         <is>
           <t>litigation</t>
         </is>
@@ -57251,7 +57167,7 @@
           <t>Maine MHDO Prescription Drug Pricing and Transparency Report (2022, covering CY2021), p.24</t>
         </is>
       </c>
-      <c r="K2045" s="20" t="inlineStr">
+      <c r="K2045" t="inlineStr">
         <is>
           <t>state_disclosure</t>
         </is>
@@ -57959,11 +57875,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A3:K3"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -57992,27 +57903,27 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Total Medicaid Overpayment</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Top Drug</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Top Drug Overpayment</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Drugs Analyzed</t>
         </is>
@@ -59111,9 +59022,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -59131,168 +59039,172 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>What this analysis covers</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>This workbook quantifies the estimated annual overpayment by Medicare Part D and Medicaid on generic drugs, compared to what the same drugs cost at Cost Plus Drugs. It covers 2,012 matched generic drugs representing 88.1% of the Cost Plus catalog.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>This workbook quantifies the estimated annual overpayment by Medicare Part D and Medicaid on generic drugs, compared to what the same drugs cost at Cost Plus Drugs. It covers 2,062 matched generic drugs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Data sources</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>•  Cost Plus Drugs prices: Cost Plus GraphQL storefront API</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>•  NADAC (National Average Drug Acquisition Cost): CMS, updated weekly. The actual price pharmacies pay to acquire each drug.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>•  Medicare Part D Spending by Drug: CMS annual dataset.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>•  Medicaid State Drug Utilization Data (SDUD): CMS quarterly dataset, broken out by state.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>•  Confirmed spread citations: federal reports including FTC Second Interim Staff Report (Jan 2025), Maine MHDO Drug Price Transparency Report, Ohio Auditor PBM Spread Report (2018), JAMA Health Forum (Mattingly et al., Oct 2023), and others. See Source Citation column.</t>
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Methodology</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>•  All comparisons are on a per-unit basis (per tablet, per mL, per gram) using the NADAC Pricing Unit as the canonical unit.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>•  Cost Plus per-unit price = (acquisition cost × 1.15 + pharmacy fee) ÷ package quantity.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>•  Overpayment = (Medicare or Medicaid price per unit − Cost Plus price per unit) × total dosage units. As of this version, Medicare Part D's overpayment is dollarized ONCE PER MOLECULE (the highest-priced strength represents the molecule; see “Part D molecule-level fix” below), not once per strength.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>•  Only generic drugs are included. Brand drug rebates are negotiated privately and never disclosed; including them would require estimating numbers that do not exist publicly.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>•  Net prices are never estimated. The "net_per_unit" field is always "not public" by design.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>•  Estimated PBM Price: where a confirmed markup percentage exists from a named government or academic source, an estimated PBM billing price is computed as NADAC acquisition cost × (1 + markup %). This is an estimate derived from a confirmed markup percentage, not a directly observed transaction price. It is labeled explicitly as estimated throughout.</t>
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Part D molecule-level fix</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>•  Medicare Part D publishes spending by generic name, not by strength -- one national Tot_Dsg_Unts/Tot_Spndng figure covers every strength of a molecule combined. Multiplying that same national figure by each strength's own per-unit gap and summing across every strength row -- the prior behavior -- counted the national total once per strength (e.g. Atorvastatin's 4 strengths each carried the full national unit count).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>•  Fixed by dollarizing once per molecule: the strength with the HIGHEST Cost Plus per-unit price represents the molecule (minimizes the gap, so the figure is a conservative floor, never inflated). Every other strength row of that molecule contributes $0. Per-strength Gap/unit stays real and visible for every row regardless.</t>
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Honest limitations</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>•  Medicare Part D spending figures are gross of manufacturer rebates. For generics, rebates are minimal; for brands, this analysis excludes them entirely.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>•  Medicaid SDUD reimbursement rates are a proxy for commercial reimbursement, not an exact equivalent.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>•  Shipping fees ($5 per order at Cost Plus) are excluded from per-unit calculations as they are per-order, not per-unit.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>•  Match confidence: 88.1% of the Cost Plus catalog matched to federal drug codes via the NIH RxNav crosswalk. Unmatched drugs are excluded.</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>•  Match confidence: matched to federal drug codes via the NIH RxNav crosswalk; unmatched drugs are excluded from this workbook.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>•  No public data gives the real strength-mix Part D dispenses at, so the highest-price-strength rule is a deliberate, documented choice, not an estimate of the true weighted-average price.</t>
         </is>
@@ -59320,27 +59232,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Source Name</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Publisher</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>What it contains</t>
         </is>
@@ -59374,27 +59286,27 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>FTC First Interim Staff Report on PBMs</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>FTC</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>ftc.gov</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Two cancer drugs, $1.6B excess revenue</t>
         </is>
@@ -59428,27 +59340,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Ohio Auditor PBM Spread Report</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Ohio Auditor of State</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>ohioauditor.gov</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>$224.8M spread on Medicaid generics</t>
         </is>
@@ -59482,27 +59394,27 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>CMS NADAC</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Weekly</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>data.medicaid.gov</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Drug acquisition costs</t>
         </is>
@@ -59536,27 +59448,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>CMS Medicaid SDUD</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Quarterly</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>data.medicaid.gov</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>State-level Medicaid drug utilization and reimbursement</t>
         </is>

</xml_diff>